<commit_message>
Optimize Agus 5 and 7 RBFNN forecast shape
</commit_message>
<xml_diff>
--- a/optimized_version/metadata/testing_daily_metrics/agus1_testing_daily_metrics.xlsx
+++ b/optimized_version/metadata/testing_daily_metrics/agus1_testing_daily_metrics.xlsx
@@ -467,7 +467,7 @@
         <v>45757</v>
       </c>
       <c r="B2" t="n">
-        <v>4.550096675554547</v>
+        <v>4.467856484336752</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -476,10 +476,10 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>1.431269310069087</v>
+        <v>1.4054</v>
       </c>
       <c r="F2" t="n">
-        <v>1.431269310069087</v>
+        <v>1.4054</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
@@ -491,7 +491,7 @@
         <v>45758</v>
       </c>
       <c r="B3" t="n">
-        <v>2.429507631931144</v>
+        <v>2.38954845879497</v>
       </c>
       <c r="C3" t="n">
         <v>24</v>
@@ -500,13 +500,13 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.7250367772559329</v>
+        <v>0.7131895833624373</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9379375465084699</v>
+        <v>0.9215928304556827</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.04752545016463317</v>
+        <v>-0.01133471561684996</v>
       </c>
       <c r="H3" t="n">
         <v>24</v>
@@ -517,7 +517,7 @@
         <v>45759</v>
       </c>
       <c r="B4" t="n">
-        <v>2.090119403324683</v>
+        <v>2.061436786036267</v>
       </c>
       <c r="C4" t="n">
         <v>24</v>
@@ -526,13 +526,13 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6301837735210855</v>
+        <v>0.6212875000194026</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8284530183379808</v>
+        <v>0.8069382158511816</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.07642997394833428</v>
+        <v>-0.02124649931490818</v>
       </c>
       <c r="H4" t="n">
         <v>24</v>
@@ -543,7 +543,7 @@
         <v>45760</v>
       </c>
       <c r="B5" t="n">
-        <v>2.255105513411784</v>
+        <v>2.259633084486148</v>
       </c>
       <c r="C5" t="n">
         <v>24</v>
@@ -552,13 +552,13 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6772666182165342</v>
+        <v>0.6792937500097013</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8775731180891762</v>
+        <v>0.8726396933991923</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.09906930126149716</v>
+        <v>-0.08674682993718608</v>
       </c>
       <c r="H5" t="n">
         <v>24</v>
@@ -569,7 +569,7 @@
         <v>45761</v>
       </c>
       <c r="B6" t="n">
-        <v>3.05514755159589</v>
+        <v>3.346787741614864</v>
       </c>
       <c r="C6" t="n">
         <v>24</v>
@@ -578,13 +578,13 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>1.144497188605119</v>
+        <v>1.258204748336489</v>
       </c>
       <c r="F6" t="n">
-        <v>2.137897781042417</v>
+        <v>2.204466611178614</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8373132680269164</v>
+        <v>0.827024213903558</v>
       </c>
       <c r="H6" t="n">
         <v>24</v>
@@ -595,7 +595,7 @@
         <v>45762</v>
       </c>
       <c r="B7" t="n">
-        <v>3.443082819152216</v>
+        <v>3.761862231896417</v>
       </c>
       <c r="C7" t="n">
         <v>24</v>
@@ -604,13 +604,13 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>1.812117244384296</v>
+        <v>1.91968024803012</v>
       </c>
       <c r="F7" t="n">
-        <v>3.080191497707655</v>
+        <v>3.078332871884333</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8570448485670049</v>
+        <v>0.8572173183454886</v>
       </c>
       <c r="H7" t="n">
         <v>24</v>
@@ -621,7 +621,7 @@
         <v>45763</v>
       </c>
       <c r="B8" t="n">
-        <v>2.427758862943838</v>
+        <v>2.450362247841603</v>
       </c>
       <c r="C8" t="n">
         <v>24</v>
@@ -630,13 +630,13 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>1.496476906185712</v>
+        <v>1.512166328454612</v>
       </c>
       <c r="F8" t="n">
-        <v>1.878203387795586</v>
+        <v>1.888884347639409</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.4651338277714845</v>
+        <v>-0.4818450445865299</v>
       </c>
       <c r="H8" t="n">
         <v>24</v>
@@ -647,7 +647,7 @@
         <v>45764</v>
       </c>
       <c r="B9" t="n">
-        <v>5.64210197342418</v>
+        <v>6.211745524735519</v>
       </c>
       <c r="C9" t="n">
         <v>24</v>
@@ -656,13 +656,13 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>2.078730852025347</v>
+        <v>2.314038092632249</v>
       </c>
       <c r="F9" t="n">
-        <v>4.820816569415689</v>
+        <v>5.12331964317877</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8630541306531115</v>
+        <v>0.8453283822898656</v>
       </c>
       <c r="H9" t="n">
         <v>24</v>
@@ -673,7 +673,7 @@
         <v>45765</v>
       </c>
       <c r="B10" t="n">
-        <v>2.681457860470941</v>
+        <v>2.643370975134389</v>
       </c>
       <c r="C10" t="n">
         <v>24</v>
@@ -682,13 +682,13 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7966931588140627</v>
+        <v>0.7851478623492173</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9551315565689398</v>
+        <v>0.9438345210398222</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.2177047820565745</v>
+        <v>-0.1890697729861175</v>
       </c>
       <c r="H10" t="n">
         <v>24</v>
@@ -699,7 +699,7 @@
         <v>45766</v>
       </c>
       <c r="B11" t="n">
-        <v>4.381480090337647</v>
+        <v>4.285245672603081</v>
       </c>
       <c r="C11" t="n">
         <v>24</v>
@@ -708,13 +708,13 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>2.046039379573507</v>
+        <v>2.004418941517368</v>
       </c>
       <c r="F11" t="n">
-        <v>4.394937943265393</v>
+        <v>4.233137657667561</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9039152947319138</v>
+        <v>0.9108598109039749</v>
       </c>
       <c r="H11" t="n">
         <v>24</v>
@@ -725,7 +725,7 @@
         <v>45767</v>
       </c>
       <c r="B12" t="n">
-        <v>2.317212379254846</v>
+        <v>2.293279057272167</v>
       </c>
       <c r="C12" t="n">
         <v>24</v>
@@ -734,13 +734,13 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>1.399302529401353</v>
+        <v>1.391485154558187</v>
       </c>
       <c r="F12" t="n">
-        <v>1.729076770922628</v>
+        <v>1.773839216404177</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1249678413670485</v>
+        <v>-0.1839682584309488</v>
       </c>
       <c r="H12" t="n">
         <v>24</v>
@@ -751,7 +751,7 @@
         <v>45768</v>
       </c>
       <c r="B13" t="n">
-        <v>6.26705181046006</v>
+        <v>6.33296654550143</v>
       </c>
       <c r="C13" t="n">
         <v>24</v>
@@ -760,13 +760,13 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>3.263303383134241</v>
+        <v>3.314300950022131</v>
       </c>
       <c r="F13" t="n">
-        <v>6.188989631870685</v>
+        <v>5.896320573404636</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.7123850638165667</v>
+        <v>-0.5542615220059743</v>
       </c>
       <c r="H13" t="n">
         <v>24</v>
@@ -777,7 +777,7 @@
         <v>45769</v>
       </c>
       <c r="B14" t="n">
-        <v>3.560168004607761</v>
+        <v>3.57914220123403</v>
       </c>
       <c r="C14" t="n">
         <v>24</v>
@@ -786,13 +786,13 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>2.082564273500743</v>
+        <v>2.095047171802136</v>
       </c>
       <c r="F14" t="n">
-        <v>2.59407600882047</v>
+        <v>2.603982992325356</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.1691892763434941</v>
+        <v>-0.1781367838966299</v>
       </c>
       <c r="H14" t="n">
         <v>24</v>
@@ -803,7 +803,7 @@
         <v>45770</v>
       </c>
       <c r="B15" t="n">
-        <v>3.547978160158011</v>
+        <v>3.727780271414478</v>
       </c>
       <c r="C15" t="n">
         <v>24</v>
@@ -812,13 +812,13 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>2.098384642867466</v>
+        <v>2.202329311149571</v>
       </c>
       <c r="F15" t="n">
-        <v>2.668876585568622</v>
+        <v>2.802529005556754</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.6520076067135552</v>
+        <v>-0.8216095391250389</v>
       </c>
       <c r="H15" t="n">
         <v>24</v>
@@ -829,7 +829,7 @@
         <v>45771</v>
       </c>
       <c r="B16" t="n">
-        <v>2.387593970170728</v>
+        <v>2.37373801137056</v>
       </c>
       <c r="C16" t="n">
         <v>24</v>
@@ -838,13 +838,13 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>1.433509338799859</v>
+        <v>1.422589947804283</v>
       </c>
       <c r="F16" t="n">
-        <v>1.842611987293778</v>
+        <v>1.770945936041948</v>
       </c>
       <c r="G16" t="n">
-        <v>0.07384526108605483</v>
+        <v>0.1444874691148536</v>
       </c>
       <c r="H16" t="n">
         <v>24</v>
@@ -855,7 +855,7 @@
         <v>45772</v>
       </c>
       <c r="B17" t="n">
-        <v>2.563966953515857</v>
+        <v>2.680897802394556</v>
       </c>
       <c r="C17" t="n">
         <v>24</v>
@@ -864,13 +864,13 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>1.524883626784532</v>
+        <v>1.591040741135319</v>
       </c>
       <c r="F17" t="n">
-        <v>1.717536919587026</v>
+        <v>1.922220366210975</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.008985245474509407</v>
+        <v>-0.2638018934322808</v>
       </c>
       <c r="H17" t="n">
         <v>24</v>
@@ -881,7 +881,7 @@
         <v>45773</v>
       </c>
       <c r="B18" t="n">
-        <v>6.282044235905391</v>
+        <v>6.230456219742294</v>
       </c>
       <c r="C18" t="n">
         <v>24</v>
@@ -890,13 +890,13 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>2.167035435684955</v>
+        <v>2.164255193049091</v>
       </c>
       <c r="F18" t="n">
-        <v>5.993652199248709</v>
+        <v>5.922376734567997</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8132515536331674</v>
+        <v>0.8176667042938686</v>
       </c>
       <c r="H18" t="n">
         <v>24</v>
@@ -907,7 +907,7 @@
         <v>45774</v>
       </c>
       <c r="B19" t="n">
-        <v>12.62360831254376</v>
+        <v>12.50392467390889</v>
       </c>
       <c r="C19" t="n">
         <v>16</v>
@@ -916,13 +916,13 @@
         <v>8</v>
       </c>
       <c r="E19" t="n">
-        <v>4.434281935981146</v>
+        <v>4.392160921739079</v>
       </c>
       <c r="F19" t="n">
-        <v>8.762293255773958</v>
+        <v>8.53207912948111</v>
       </c>
       <c r="G19" t="n">
-        <v>0.8509007749173579</v>
+        <v>0.8586325033821561</v>
       </c>
       <c r="H19" t="n">
         <v>24</v>
@@ -933,7 +933,7 @@
         <v>45775</v>
       </c>
       <c r="B20" t="n">
-        <v>2.55278490820086</v>
+        <v>2.4358238741253</v>
       </c>
       <c r="C20" t="n">
         <v>24</v>
@@ -942,13 +942,13 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>1.539962858250633</v>
+        <v>1.471733979046708</v>
       </c>
       <c r="F20" t="n">
-        <v>1.850068920468198</v>
+        <v>1.762274702857972</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.4286138772422434</v>
+        <v>-0.2962425210921837</v>
       </c>
       <c r="H20" t="n">
         <v>24</v>
@@ -959,7 +959,7 @@
         <v>45776</v>
       </c>
       <c r="B21" t="n">
-        <v>2.803500662469447</v>
+        <v>3.010814276399258</v>
       </c>
       <c r="C21" t="n">
         <v>24</v>
@@ -968,13 +968,13 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>1.648903288229875</v>
+        <v>1.774075601912893</v>
       </c>
       <c r="F21" t="n">
-        <v>2.043101775078928</v>
+        <v>2.213280672389437</v>
       </c>
       <c r="G21" t="n">
-        <v>0.02956247262494871</v>
+        <v>-0.13883436411725</v>
       </c>
       <c r="H21" t="n">
         <v>24</v>
@@ -985,7 +985,7 @@
         <v>45777</v>
       </c>
       <c r="B22" t="n">
-        <v>2.529366661244516</v>
+        <v>2.351111226446162</v>
       </c>
       <c r="C22" t="n">
         <v>24</v>
@@ -994,13 +994,13 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>1.51113032167814</v>
+        <v>1.402367647366917</v>
       </c>
       <c r="F22" t="n">
-        <v>1.754063477581248</v>
+        <v>1.73151199365775</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.1317792676608842</v>
+        <v>-0.1028644313974549</v>
       </c>
       <c r="H22" t="n">
         <v>24</v>
@@ -1011,7 +1011,7 @@
         <v>45778</v>
       </c>
       <c r="B23" t="n">
-        <v>2.537195071974848</v>
+        <v>2.813387022412368</v>
       </c>
       <c r="C23" t="n">
         <v>24</v>
@@ -1020,13 +1020,13 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>1.489325206863089</v>
+        <v>1.653468144700775</v>
       </c>
       <c r="F23" t="n">
-        <v>1.788450637357565</v>
+        <v>1.851831450701776</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1064310372682264</v>
+        <v>-0.1862421344488616</v>
       </c>
       <c r="H23" t="n">
         <v>24</v>
@@ -1037,7 +1037,7 @@
         <v>45779</v>
       </c>
       <c r="B24" t="n">
-        <v>2.368147966795133</v>
+        <v>2.677879443672064</v>
       </c>
       <c r="C24" t="n">
         <v>24</v>
@@ -1046,13 +1046,13 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>1.405009700878727</v>
+        <v>1.592771021769755</v>
       </c>
       <c r="F24" t="n">
-        <v>1.740648833532738</v>
+        <v>2.113576578346412</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.04387929051541062</v>
+        <v>-0.5390896945209056</v>
       </c>
       <c r="H24" t="n">
         <v>24</v>
@@ -1063,7 +1063,7 @@
         <v>45780</v>
       </c>
       <c r="B25" t="n">
-        <v>5.694188645847778</v>
+        <v>5.578460245004218</v>
       </c>
       <c r="C25" t="n">
         <v>24</v>
@@ -1072,13 +1072,13 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>3.198500725459299</v>
+        <v>3.136171309673886</v>
       </c>
       <c r="F25" t="n">
-        <v>4.261079523064178</v>
+        <v>4.270121503867492</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2237962122999551</v>
+        <v>0.2204985192019941</v>
       </c>
       <c r="H25" t="n">
         <v>24</v>
@@ -1089,7 +1089,7 @@
         <v>45781</v>
       </c>
       <c r="B26" t="n">
-        <v>4.921798727528617</v>
+        <v>5.041695327124013</v>
       </c>
       <c r="C26" t="n">
         <v>24</v>
@@ -1098,13 +1098,13 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>2.726107643616437</v>
+        <v>2.798550175143729</v>
       </c>
       <c r="F26" t="n">
-        <v>3.829989665815641</v>
+        <v>3.789088018029995</v>
       </c>
       <c r="G26" t="n">
-        <v>0.3878836956118419</v>
+        <v>0.4008878449876766</v>
       </c>
       <c r="H26" t="n">
         <v>24</v>
@@ -1115,7 +1115,7 @@
         <v>45782</v>
       </c>
       <c r="B27" t="n">
-        <v>1.505664641269149</v>
+        <v>1.765560291751407</v>
       </c>
       <c r="C27" t="n">
         <v>24</v>
@@ -1124,13 +1124,13 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>0.9054406856623339</v>
+        <v>1.064030478394938</v>
       </c>
       <c r="F27" t="n">
-        <v>1.07864635503005</v>
+        <v>1.334411232468763</v>
       </c>
       <c r="G27" t="n">
-        <v>0.08238255049065446</v>
+        <v>-0.4043743252043166</v>
       </c>
       <c r="H27" t="n">
         <v>24</v>
@@ -1141,7 +1141,7 @@
         <v>45783</v>
       </c>
       <c r="B28" t="n">
-        <v>2.186419501753831</v>
+        <v>2.569706480757909</v>
       </c>
       <c r="C28" t="n">
         <v>24</v>
@@ -1150,13 +1150,13 @@
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>1.276395959274356</v>
+        <v>1.51171136039164</v>
       </c>
       <c r="F28" t="n">
-        <v>1.936560862121522</v>
+        <v>2.236660716211738</v>
       </c>
       <c r="G28" t="n">
-        <v>-0.1045975875914258</v>
+        <v>-0.4734724138404827</v>
       </c>
       <c r="H28" t="n">
         <v>24</v>
@@ -1167,7 +1167,7 @@
         <v>45784</v>
       </c>
       <c r="B29" t="n">
-        <v>24.1126409869719</v>
+        <v>23.92016065802341</v>
       </c>
       <c r="C29" t="n">
         <v>21</v>
@@ -1176,13 +1176,13 @@
         <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>6.039555367398154</v>
+        <v>5.967237402676905</v>
       </c>
       <c r="F29" t="n">
-        <v>12.97600177973607</v>
+        <v>12.93911824174375</v>
       </c>
       <c r="G29" t="n">
-        <v>0.6471157364230082</v>
+        <v>0.6491189917072946</v>
       </c>
       <c r="H29" t="n">
         <v>24</v>
@@ -1193,7 +1193,7 @@
         <v>45785</v>
       </c>
       <c r="B30" t="n">
-        <v>2.556519125744855</v>
+        <v>2.581841172879298</v>
       </c>
       <c r="C30" t="n">
         <v>24</v>
@@ -1202,13 +1202,13 @@
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>1.534208852693528</v>
+        <v>1.547290475831694</v>
       </c>
       <c r="F30" t="n">
-        <v>1.787424613699295</v>
+        <v>1.880480764405346</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.2585482917246731</v>
+        <v>-0.3930034981280741</v>
       </c>
       <c r="H30" t="n">
         <v>24</v>
@@ -1219,7 +1219,7 @@
         <v>45786</v>
       </c>
       <c r="B31" t="n">
-        <v>1.509117845626917</v>
+        <v>1.877176074887886</v>
       </c>
       <c r="C31" t="n">
         <v>24</v>
@@ -1228,13 +1228,13 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>0.9108697398364104</v>
+        <v>1.132479318313231</v>
       </c>
       <c r="F31" t="n">
-        <v>1.257794948326728</v>
+        <v>1.402130453841408</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1593636625891777</v>
+        <v>-0.4407108815657961</v>
       </c>
       <c r="H31" t="n">
         <v>24</v>
@@ -1245,7 +1245,7 @@
         <v>45787</v>
       </c>
       <c r="B32" t="n">
-        <v>2.268887535181495</v>
+        <v>2.356620121101336</v>
       </c>
       <c r="C32" t="n">
         <v>24</v>
@@ -1254,13 +1254,13 @@
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>1.357721157888367</v>
+        <v>1.412558756147979</v>
       </c>
       <c r="F32" t="n">
-        <v>1.655265432210508</v>
+        <v>1.923721455756158</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2518431225577253</v>
+        <v>-0.6908262992469776</v>
       </c>
       <c r="H32" t="n">
         <v>24</v>
@@ -1271,7 +1271,7 @@
         <v>45788</v>
       </c>
       <c r="B33" t="n">
-        <v>2.457402282249208</v>
+        <v>2.779676210591381</v>
       </c>
       <c r="C33" t="n">
         <v>24</v>
@@ -1280,13 +1280,13 @@
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>1.470301664929917</v>
+        <v>1.654579535269344</v>
       </c>
       <c r="F33" t="n">
-        <v>1.855780120864283</v>
+        <v>2.077339187337514</v>
       </c>
       <c r="G33" t="n">
-        <v>0.2329559168819427</v>
+        <v>0.03887003962679036</v>
       </c>
       <c r="H33" t="n">
         <v>24</v>
@@ -1297,7 +1297,7 @@
         <v>45789</v>
       </c>
       <c r="B34" t="n">
-        <v>2.984880806141689</v>
+        <v>2.819180613378666</v>
       </c>
       <c r="C34" t="n">
         <v>24</v>
@@ -1306,13 +1306,13 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>1.82697961147827</v>
+        <v>1.726897940974263</v>
       </c>
       <c r="F34" t="n">
-        <v>2.164599737866731</v>
+        <v>2.068610728219574</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.166560283389839</v>
+        <v>-0.06539223889431933</v>
       </c>
       <c r="H34" t="n">
         <v>24</v>
@@ -1323,7 +1323,7 @@
         <v>45790</v>
       </c>
       <c r="B35" t="n">
-        <v>2.472079875304737</v>
+        <v>2.843292000401497</v>
       </c>
       <c r="C35" t="n">
         <v>24</v>
@@ -1332,13 +1332,13 @@
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>1.48658837070846</v>
+        <v>1.71839940241066</v>
       </c>
       <c r="F35" t="n">
-        <v>1.85383504164475</v>
+        <v>2.169403128295943</v>
       </c>
       <c r="G35" t="n">
-        <v>-0.1265658601425181</v>
+        <v>-0.5427478013618268</v>
       </c>
       <c r="H35" t="n">
         <v>24</v>
@@ -1349,7 +1349,7 @@
         <v>45791</v>
       </c>
       <c r="B36" t="n">
-        <v>5.017195388524684</v>
+        <v>4.920832409758938</v>
       </c>
       <c r="C36" t="n">
         <v>24</v>
@@ -1358,13 +1358,13 @@
         <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>3.071126738770527</v>
+        <v>2.996603781427188</v>
       </c>
       <c r="F36" t="n">
-        <v>4.178065587686278</v>
+        <v>4.097557806466368</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1182637598032722</v>
+        <v>0.1519169903596167</v>
       </c>
       <c r="H36" t="n">
         <v>24</v>
@@ -1375,7 +1375,7 @@
         <v>45792</v>
       </c>
       <c r="B37" t="n">
-        <v>1.902004308082443</v>
+        <v>1.904931855786345</v>
       </c>
       <c r="C37" t="n">
         <v>24</v>
@@ -1384,13 +1384,13 @@
         <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>1.146980185905935</v>
+        <v>1.151067532550549</v>
       </c>
       <c r="F37" t="n">
-        <v>1.47746143135108</v>
+        <v>1.54868547814116</v>
       </c>
       <c r="G37" t="n">
-        <v>-0.05327040118325832</v>
+        <v>-0.157268219373107</v>
       </c>
       <c r="H37" t="n">
         <v>24</v>
@@ -1401,7 +1401,7 @@
         <v>45793</v>
       </c>
       <c r="B38" t="n">
-        <v>2.00418157941375</v>
+        <v>2.442064258901516</v>
       </c>
       <c r="C38" t="n">
         <v>24</v>
@@ -1410,13 +1410,13 @@
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>1.184614642549784</v>
+        <v>1.445258299031825</v>
       </c>
       <c r="F38" t="n">
-        <v>1.45425996718101</v>
+        <v>1.692431104389158</v>
       </c>
       <c r="G38" t="n">
-        <v>0.1015811775057353</v>
+        <v>-0.2167931071849942</v>
       </c>
       <c r="H38" t="n">
         <v>24</v>
@@ -1427,7 +1427,7 @@
         <v>45794</v>
       </c>
       <c r="B39" t="n">
-        <v>3.020019399029628</v>
+        <v>3.171078262710949</v>
       </c>
       <c r="C39" t="n">
         <v>24</v>
@@ -1436,13 +1436,13 @@
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>1.786031907287829</v>
+        <v>1.882291622689476</v>
       </c>
       <c r="F39" t="n">
-        <v>2.007401767514614</v>
+        <v>2.172445682463222</v>
       </c>
       <c r="G39" t="n">
-        <v>-0.003229567757726093</v>
+        <v>-0.1749775595570988</v>
       </c>
       <c r="H39" t="n">
         <v>24</v>
@@ -1453,7 +1453,7 @@
         <v>45795</v>
       </c>
       <c r="B40" t="n">
-        <v>2.406508530169742</v>
+        <v>2.214760177848838</v>
       </c>
       <c r="C40" t="n">
         <v>24</v>
@@ -1462,13 +1462,13 @@
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>1.444946430532398</v>
+        <v>1.332239172288027</v>
       </c>
       <c r="F40" t="n">
-        <v>1.766604375712697</v>
+        <v>1.613970745748269</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.4144002621411047</v>
+        <v>-0.180551783726645</v>
       </c>
       <c r="H40" t="n">
         <v>24</v>
@@ -1479,7 +1479,7 @@
         <v>45796</v>
       </c>
       <c r="B41" t="n">
-        <v>2.902608704771703</v>
+        <v>2.935221720136002</v>
       </c>
       <c r="C41" t="n">
         <v>24</v>
@@ -1488,13 +1488,13 @@
         <v>0</v>
       </c>
       <c r="E41" t="n">
-        <v>1.71901353095726</v>
+        <v>1.739076000605684</v>
       </c>
       <c r="F41" t="n">
-        <v>1.983179212431498</v>
+        <v>2.002909434029713</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.002132774110688684</v>
+        <v>-0.0221719685100652</v>
       </c>
       <c r="H41" t="n">
         <v>24</v>
@@ -1505,7 +1505,7 @@
         <v>45797</v>
       </c>
       <c r="B42" t="n">
-        <v>3.015789476865694</v>
+        <v>3.063021877235351</v>
       </c>
       <c r="C42" t="n">
         <v>24</v>
@@ -1514,13 +1514,13 @@
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>1.762706273011633</v>
+        <v>1.796122896470657</v>
       </c>
       <c r="F42" t="n">
-        <v>2.359928122120088</v>
+        <v>2.415049071887311</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.585138212343681</v>
+        <v>-0.660051279397839</v>
       </c>
       <c r="H42" t="n">
         <v>24</v>
@@ -1531,7 +1531,7 @@
         <v>45798</v>
       </c>
       <c r="B43" t="n">
-        <v>3.084071957798094</v>
+        <v>3.10476589781103</v>
       </c>
       <c r="C43" t="n">
         <v>24</v>
@@ -1540,13 +1540,13 @@
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>1.791748253364632</v>
+        <v>1.803912864133621</v>
       </c>
       <c r="F43" t="n">
-        <v>2.339678252819333</v>
+        <v>2.318993557255856</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.8256960155832613</v>
+        <v>-0.7935573795612736</v>
       </c>
       <c r="H43" t="n">
         <v>24</v>
@@ -1557,7 +1557,7 @@
         <v>45799</v>
       </c>
       <c r="B44" t="n">
-        <v>3.028455651554085</v>
+        <v>2.874052376911358</v>
       </c>
       <c r="C44" t="n">
         <v>24</v>
@@ -1566,13 +1566,13 @@
         <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>1.754571564253195</v>
+        <v>1.661202295994799</v>
       </c>
       <c r="F44" t="n">
-        <v>2.414200850732573</v>
+        <v>2.416268171704061</v>
       </c>
       <c r="G44" t="n">
-        <v>0.03931984960495438</v>
+        <v>0.03767385187570238</v>
       </c>
       <c r="H44" t="n">
         <v>24</v>
@@ -1583,7 +1583,7 @@
         <v>45800</v>
       </c>
       <c r="B45" t="n">
-        <v>5.257875035756411</v>
+        <v>5.197082090144351</v>
       </c>
       <c r="C45" t="n">
         <v>24</v>
@@ -1592,13 +1592,13 @@
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>2.831338837662177</v>
+        <v>2.798712018135034</v>
       </c>
       <c r="F45" t="n">
-        <v>3.411154567241764</v>
+        <v>3.464048491803542</v>
       </c>
       <c r="G45" t="n">
-        <v>0.1302703340650457</v>
+        <v>0.1030888723675984</v>
       </c>
       <c r="H45" t="n">
         <v>24</v>
@@ -1609,7 +1609,7 @@
         <v>45801</v>
       </c>
       <c r="B46" t="n">
-        <v>4.0196577155379</v>
+        <v>4.395321915645887</v>
       </c>
       <c r="C46" t="n">
         <v>24</v>
@@ -1618,13 +1618,13 @@
         <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>2.232884777948533</v>
+        <v>2.447477880622396</v>
       </c>
       <c r="F46" t="n">
-        <v>2.981432079899907</v>
+        <v>3.099444710904937</v>
       </c>
       <c r="G46" t="n">
-        <v>0.5506094175677065</v>
+        <v>0.5143292884990571</v>
       </c>
       <c r="H46" t="n">
         <v>24</v>
@@ -1635,7 +1635,7 @@
         <v>45802</v>
       </c>
       <c r="B47" t="n">
-        <v>3.257965484662392</v>
+        <v>3.335470504536287</v>
       </c>
       <c r="C47" t="n">
         <v>24</v>
@@ -1644,13 +1644,13 @@
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>1.889171396750187</v>
+        <v>1.9409680257564</v>
       </c>
       <c r="F47" t="n">
-        <v>2.500306546682712</v>
+        <v>2.563929810529029</v>
       </c>
       <c r="G47" t="n">
-        <v>-0.6537433753148221</v>
+        <v>-0.738977108893865</v>
       </c>
       <c r="H47" t="n">
         <v>24</v>
@@ -1661,7 +1661,7 @@
         <v>45803</v>
       </c>
       <c r="B48" t="n">
-        <v>2.573663412540167</v>
+        <v>2.65462515777342</v>
       </c>
       <c r="C48" t="n">
         <v>24</v>
@@ -1670,13 +1670,13 @@
         <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>1.533210961360843</v>
+        <v>1.582285047554705</v>
       </c>
       <c r="F48" t="n">
-        <v>2.043223346197538</v>
+        <v>2.266977449527673</v>
       </c>
       <c r="G48" t="n">
-        <v>-0.6128290864378283</v>
+        <v>-0.9854139210043562</v>
       </c>
       <c r="H48" t="n">
         <v>24</v>
@@ -1687,7 +1687,7 @@
         <v>45804</v>
       </c>
       <c r="B49" t="n">
-        <v>2.931526886187902</v>
+        <v>3.231499197688319</v>
       </c>
       <c r="C49" t="n">
         <v>24</v>
@@ -1696,13 +1696,13 @@
         <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>1.722013852251397</v>
+        <v>1.899611136981617</v>
       </c>
       <c r="F49" t="n">
-        <v>2.055721470527377</v>
+        <v>2.343468835754719</v>
       </c>
       <c r="G49" t="n">
-        <v>-0.3127424858397359</v>
+        <v>-0.7059620367344981</v>
       </c>
       <c r="H49" t="n">
         <v>24</v>
@@ -1713,7 +1713,7 @@
         <v>45805</v>
       </c>
       <c r="B50" t="n">
-        <v>3.133116850653578</v>
+        <v>2.806581606247073</v>
       </c>
       <c r="C50" t="n">
         <v>24</v>
@@ -1722,13 +1722,13 @@
         <v>0</v>
       </c>
       <c r="E50" t="n">
-        <v>1.870595479996696</v>
+        <v>1.679055144760431</v>
       </c>
       <c r="F50" t="n">
-        <v>2.203049735641749</v>
+        <v>2.013722721276028</v>
       </c>
       <c r="G50" t="n">
-        <v>-0.508576089195055</v>
+        <v>-0.2604277522189757</v>
       </c>
       <c r="H50" t="n">
         <v>24</v>
@@ -1739,7 +1739,7 @@
         <v>45806</v>
       </c>
       <c r="B51" t="n">
-        <v>3.095785688988121</v>
+        <v>3.142080097722522</v>
       </c>
       <c r="C51" t="n">
         <v>24</v>
@@ -1748,13 +1748,13 @@
         <v>0</v>
       </c>
       <c r="E51" t="n">
-        <v>1.804937138514185</v>
+        <v>1.83066627889736</v>
       </c>
       <c r="F51" t="n">
-        <v>2.395207994845577</v>
+        <v>2.49004234027597</v>
       </c>
       <c r="G51" t="n">
-        <v>-0.3810565338851648</v>
+        <v>-0.492582877935742</v>
       </c>
       <c r="H51" t="n">
         <v>24</v>
@@ -1765,7 +1765,7 @@
         <v>45807</v>
       </c>
       <c r="B52" t="n">
-        <v>2.121743224402911</v>
+        <v>2.00607467373345</v>
       </c>
       <c r="C52" t="n">
         <v>24</v>
@@ -1774,13 +1774,13 @@
         <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>1.256775717312703</v>
+        <v>1.192817336229209</v>
       </c>
       <c r="F52" t="n">
-        <v>1.445261467910204</v>
+        <v>1.374857431386889</v>
       </c>
       <c r="G52" t="n">
-        <v>-0.04573513388564199</v>
+        <v>0.0536665702000082</v>
       </c>
       <c r="H52" t="n">
         <v>24</v>
@@ -1791,7 +1791,7 @@
         <v>45808</v>
       </c>
       <c r="B53" t="n">
-        <v>2.003818766408649</v>
+        <v>2.355343949560957</v>
       </c>
       <c r="C53" t="n">
         <v>24</v>
@@ -1800,13 +1800,13 @@
         <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>1.153216401240985</v>
+        <v>1.355750303035429</v>
       </c>
       <c r="F53" t="n">
-        <v>1.62588752639157</v>
+        <v>1.792925270882958</v>
       </c>
       <c r="G53" t="n">
-        <v>0.1281387332939832</v>
+        <v>-0.0602072330606267</v>
       </c>
       <c r="H53" t="n">
         <v>24</v>
@@ -1817,7 +1817,7 @@
         <v>45809</v>
       </c>
       <c r="B54" t="n">
-        <v>2.13425430207076</v>
+        <v>2.068185485073321</v>
       </c>
       <c r="C54" t="n">
         <v>24</v>
@@ -1826,13 +1826,13 @@
         <v>0</v>
       </c>
       <c r="E54" t="n">
-        <v>1.245256981311222</v>
+        <v>1.210492671368059</v>
       </c>
       <c r="F54" t="n">
-        <v>1.546851551299846</v>
+        <v>1.512867217900863</v>
       </c>
       <c r="G54" t="n">
-        <v>-0.1218267930908246</v>
+        <v>-0.07307520133526757</v>
       </c>
       <c r="H54" t="n">
         <v>24</v>
@@ -1843,7 +1843,7 @@
         <v>45810</v>
       </c>
       <c r="B55" t="n">
-        <v>1.440102882329618</v>
+        <v>1.564251575940094</v>
       </c>
       <c r="C55" t="n">
         <v>24</v>
@@ -1852,13 +1852,13 @@
         <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>0.863277242999879</v>
+        <v>0.9424179381354983</v>
       </c>
       <c r="F55" t="n">
-        <v>1.211127102041732</v>
+        <v>1.267148366618033</v>
       </c>
       <c r="G55" t="n">
-        <v>0.09332597880571991</v>
+        <v>0.007508804041526762</v>
       </c>
       <c r="H55" t="n">
         <v>24</v>
@@ -1869,7 +1869,7 @@
         <v>45811</v>
       </c>
       <c r="B56" t="n">
-        <v>1.831532017932932</v>
+        <v>1.919894131805276</v>
       </c>
       <c r="C56" t="n">
         <v>24</v>
@@ -1878,13 +1878,13 @@
         <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>1.093678268489295</v>
+        <v>1.150839878729013</v>
       </c>
       <c r="F56" t="n">
-        <v>1.405705095083477</v>
+        <v>1.581682932599668</v>
       </c>
       <c r="G56" t="n">
-        <v>0.368737949335303</v>
+        <v>0.2007914883669337</v>
       </c>
       <c r="H56" t="n">
         <v>24</v>
@@ -1895,7 +1895,7 @@
         <v>45812</v>
       </c>
       <c r="B57" t="n">
-        <v>2.70827551964156</v>
+        <v>2.809123238713227</v>
       </c>
       <c r="C57" t="n">
         <v>24</v>
@@ -1904,13 +1904,13 @@
         <v>0</v>
       </c>
       <c r="E57" t="n">
-        <v>1.593526010477453</v>
+        <v>1.657146029872393</v>
       </c>
       <c r="F57" t="n">
-        <v>2.225495394905422</v>
+        <v>2.259220647882318</v>
       </c>
       <c r="G57" t="n">
-        <v>-0.5757017709403012</v>
+        <v>-0.6238201278829847</v>
       </c>
       <c r="H57" t="n">
         <v>24</v>
@@ -1921,7 +1921,7 @@
         <v>45813</v>
       </c>
       <c r="B58" t="n">
-        <v>2.884149262582264</v>
+        <v>2.975695708913443</v>
       </c>
       <c r="C58" t="n">
         <v>24</v>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>1.681930019978772</v>
+        <v>1.737290503456282</v>
       </c>
       <c r="F58" t="n">
-        <v>2.237801348596428</v>
+        <v>2.269452018387049</v>
       </c>
       <c r="G58" t="n">
-        <v>-0.2553024499679422</v>
+        <v>-0.2910626706938508</v>
       </c>
       <c r="H58" t="n">
         <v>24</v>
@@ -1947,7 +1947,7 @@
         <v>45814</v>
       </c>
       <c r="B59" t="n">
-        <v>1.576143384208073</v>
+        <v>1.585529994555606</v>
       </c>
       <c r="C59" t="n">
         <v>24</v>
@@ -1956,13 +1956,13 @@
         <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>0.9328517266389417</v>
+        <v>0.9414762617511047</v>
       </c>
       <c r="F59" t="n">
-        <v>1.209096781782964</v>
+        <v>1.118612496626781</v>
       </c>
       <c r="G59" t="n">
-        <v>-0.03999363053617255</v>
+        <v>0.1098403945720061</v>
       </c>
       <c r="H59" t="n">
         <v>24</v>
@@ -1973,7 +1973,7 @@
         <v>45815</v>
       </c>
       <c r="B60" t="n">
-        <v>20.86181843507563</v>
+        <v>20.68694722314049</v>
       </c>
       <c r="C60" t="n">
         <v>11</v>
@@ -1982,13 +1982,13 @@
         <v>13</v>
       </c>
       <c r="E60" t="n">
-        <v>6.441438515281366</v>
+        <v>6.397583459047515</v>
       </c>
       <c r="F60" t="n">
-        <v>14.96042203285764</v>
+        <v>14.92001682912267</v>
       </c>
       <c r="G60" t="n">
-        <v>0.6925035868640614</v>
+        <v>0.6941623204437859</v>
       </c>
       <c r="H60" t="n">
         <v>24</v>
@@ -1999,7 +1999,7 @@
         <v>45816</v>
       </c>
       <c r="B61" t="n">
-        <v>3.673508680376615</v>
+        <v>3.826870040050155</v>
       </c>
       <c r="C61" t="n">
         <v>24</v>
@@ -2008,13 +2008,13 @@
         <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>2.047490862547819</v>
+        <v>2.12779544642643</v>
       </c>
       <c r="F61" t="n">
-        <v>3.479608196389915</v>
+        <v>3.29227953195391</v>
       </c>
       <c r="G61" t="n">
-        <v>0.6449523216781515</v>
+        <v>0.6821520675370378</v>
       </c>
       <c r="H61" t="n">
         <v>24</v>
@@ -2025,7 +2025,7 @@
         <v>45817</v>
       </c>
       <c r="B62" t="n">
-        <v>2.697263445404137</v>
+        <v>2.391569682601509</v>
       </c>
       <c r="C62" t="n">
         <v>24</v>
@@ -2034,13 +2034,13 @@
         <v>0</v>
       </c>
       <c r="E62" t="n">
-        <v>1.59705895982719</v>
+        <v>1.418224258058654</v>
       </c>
       <c r="F62" t="n">
-        <v>1.866627878322176</v>
+        <v>1.70449451522919</v>
       </c>
       <c r="G62" t="n">
-        <v>-0.5654968324781702</v>
+        <v>-0.3053528263146281</v>
       </c>
       <c r="H62" t="n">
         <v>24</v>
@@ -2051,7 +2051,7 @@
         <v>45818</v>
       </c>
       <c r="B63" t="n">
-        <v>2.811448907506152</v>
+        <v>2.824902874444087</v>
       </c>
       <c r="C63" t="n">
         <v>24</v>
@@ -2060,13 +2060,13 @@
         <v>0</v>
       </c>
       <c r="E63" t="n">
-        <v>1.661506038570405</v>
+        <v>1.669812497506198</v>
       </c>
       <c r="F63" t="n">
-        <v>2.190580609985881</v>
+        <v>2.195169264247268</v>
       </c>
       <c r="G63" t="n">
-        <v>-0.5124501581201837</v>
+        <v>-0.5187931154421024</v>
       </c>
       <c r="H63" t="n">
         <v>24</v>
@@ -2077,7 +2077,7 @@
         <v>45819</v>
       </c>
       <c r="B64" t="n">
-        <v>2.696988096591077</v>
+        <v>2.531924647551394</v>
       </c>
       <c r="C64" t="n">
         <v>24</v>
@@ -2086,13 +2086,13 @@
         <v>0</v>
       </c>
       <c r="E64" t="n">
-        <v>1.583245490664475</v>
+        <v>1.487970756224411</v>
       </c>
       <c r="F64" t="n">
-        <v>1.96210742721748</v>
+        <v>1.87502096105178</v>
       </c>
       <c r="G64" t="n">
-        <v>-0.1675624700268974</v>
+        <v>-0.06621998211886493</v>
       </c>
       <c r="H64" t="n">
         <v>24</v>
@@ -2103,7 +2103,7 @@
         <v>45820</v>
       </c>
       <c r="B65" t="n">
-        <v>3.637181863997897</v>
+        <v>3.620065661349341</v>
       </c>
       <c r="C65" t="n">
         <v>24</v>
@@ -2112,13 +2112,13 @@
         <v>0</v>
       </c>
       <c r="E65" t="n">
-        <v>2.092635949653024</v>
+        <v>2.080965370183643</v>
       </c>
       <c r="F65" t="n">
-        <v>2.718823593140656</v>
+        <v>2.685708100579645</v>
       </c>
       <c r="G65" t="n">
-        <v>-0.950739346446571</v>
+        <v>-0.9035084192827099</v>
       </c>
       <c r="H65" t="n">
         <v>24</v>
@@ -2129,7 +2129,7 @@
         <v>45821</v>
       </c>
       <c r="B66" t="n">
-        <v>4.637613668475185</v>
+        <v>3.900093721984035</v>
       </c>
       <c r="C66" t="n">
         <v>24</v>
@@ -2138,13 +2138,13 @@
         <v>0</v>
       </c>
       <c r="E66" t="n">
-        <v>2.514652248676378</v>
+        <v>2.119462791766862</v>
       </c>
       <c r="F66" t="n">
-        <v>3.535441165673149</v>
+        <v>3.115533666762563</v>
       </c>
       <c r="G66" t="n">
-        <v>0.1938343265342615</v>
+        <v>0.3739601619704793</v>
       </c>
       <c r="H66" t="n">
         <v>24</v>
@@ -2155,7 +2155,7 @@
         <v>45822</v>
       </c>
       <c r="B67" t="n">
-        <v>2.962455908734154</v>
+        <v>2.830235744112805</v>
       </c>
       <c r="C67" t="n">
         <v>24</v>
@@ -2164,13 +2164,13 @@
         <v>0</v>
       </c>
       <c r="E67" t="n">
-        <v>1.72212232866833</v>
+        <v>1.644676571447628</v>
       </c>
       <c r="F67" t="n">
-        <v>2.029878197753717</v>
+        <v>2.04717492259312</v>
       </c>
       <c r="G67" t="n">
-        <v>-0.460958342662348</v>
+        <v>-0.4859622638516161</v>
       </c>
       <c r="H67" t="n">
         <v>24</v>
@@ -2181,7 +2181,7 @@
         <v>45823</v>
       </c>
       <c r="B68" t="n">
-        <v>2.354865434229934</v>
+        <v>2.339188303441897</v>
       </c>
       <c r="C68" t="n">
         <v>24</v>
@@ -2190,13 +2190,13 @@
         <v>0</v>
       </c>
       <c r="E68" t="n">
-        <v>1.368818540055428</v>
+        <v>1.365355458277769</v>
       </c>
       <c r="F68" t="n">
-        <v>1.748250527029733</v>
+        <v>1.670092013095616</v>
       </c>
       <c r="G68" t="n">
-        <v>-0.09024916414034956</v>
+        <v>0.005054653932805575</v>
       </c>
       <c r="H68" t="n">
         <v>24</v>
@@ -2207,7 +2207,7 @@
         <v>45824</v>
       </c>
       <c r="B69" t="n">
-        <v>4.486093384467754</v>
+        <v>4.376003182008557</v>
       </c>
       <c r="C69" t="n">
         <v>24</v>
@@ -2216,13 +2216,13 @@
         <v>0</v>
       </c>
       <c r="E69" t="n">
-        <v>2.568586144425119</v>
+        <v>2.506175669727625</v>
       </c>
       <c r="F69" t="n">
-        <v>3.479695651621593</v>
+        <v>3.302103410577084</v>
       </c>
       <c r="G69" t="n">
-        <v>-0.8938421442146129</v>
+        <v>-0.7054641529756767</v>
       </c>
       <c r="H69" t="n">
         <v>24</v>
@@ -2233,7 +2233,7 @@
         <v>45825</v>
       </c>
       <c r="B70" t="n">
-        <v>2.847456756117295</v>
+        <v>2.869653058454626</v>
       </c>
       <c r="C70" t="n">
         <v>24</v>
@@ -2242,13 +2242,13 @@
         <v>0</v>
       </c>
       <c r="E70" t="n">
-        <v>1.648303452346804</v>
+        <v>1.663025864916747</v>
       </c>
       <c r="F70" t="n">
-        <v>2.160438984058251</v>
+        <v>2.092255144192158</v>
       </c>
       <c r="G70" t="n">
-        <v>-0.02647880850226425</v>
+        <v>0.03729048129464929</v>
       </c>
       <c r="H70" t="n">
         <v>24</v>
@@ -2259,7 +2259,7 @@
         <v>45826</v>
       </c>
       <c r="B71" t="n">
-        <v>1.603379738360398</v>
+        <v>1.380962458591972</v>
       </c>
       <c r="C71" t="n">
         <v>24</v>
@@ -2268,13 +2268,13 @@
         <v>0</v>
       </c>
       <c r="E71" t="n">
-        <v>0.9381820126714198</v>
+        <v>0.8072283323158507</v>
       </c>
       <c r="F71" t="n">
-        <v>1.251814876291736</v>
+        <v>1.066942891318711</v>
       </c>
       <c r="G71" t="n">
-        <v>-0.4290142351459307</v>
+        <v>-0.03809879479424838</v>
       </c>
       <c r="H71" t="n">
         <v>24</v>
@@ -2285,7 +2285,7 @@
         <v>45827</v>
       </c>
       <c r="B72" t="n">
-        <v>3.828028198755054</v>
+        <v>3.651825044473794</v>
       </c>
       <c r="C72" t="n">
         <v>24</v>
@@ -2294,13 +2294,13 @@
         <v>0</v>
       </c>
       <c r="E72" t="n">
-        <v>2.199128985318942</v>
+        <v>2.09720692623454</v>
       </c>
       <c r="F72" t="n">
-        <v>2.836729608397478</v>
+        <v>2.814629371274652</v>
       </c>
       <c r="G72" t="n">
-        <v>-0.9006546394001416</v>
+        <v>-0.8711549695751628</v>
       </c>
       <c r="H72" t="n">
         <v>24</v>
@@ -2311,7 +2311,7 @@
         <v>45828</v>
       </c>
       <c r="B73" t="n">
-        <v>3.256926950262221</v>
+        <v>3.621509037589126</v>
       </c>
       <c r="C73" t="n">
         <v>24</v>
@@ -2320,13 +2320,13 @@
         <v>0</v>
       </c>
       <c r="E73" t="n">
-        <v>1.857995340906005</v>
+        <v>2.072607821503597</v>
       </c>
       <c r="F73" t="n">
-        <v>2.476134072943412</v>
+        <v>2.7021433717662</v>
       </c>
       <c r="G73" t="n">
-        <v>0.1789661067725624</v>
+        <v>0.02224611631545248</v>
       </c>
       <c r="H73" t="n">
         <v>24</v>
@@ -2337,7 +2337,7 @@
         <v>45829</v>
       </c>
       <c r="B74" t="n">
-        <v>3.218623290185808</v>
+        <v>3.288166038636427</v>
       </c>
       <c r="C74" t="n">
         <v>24</v>
@@ -2346,13 +2346,13 @@
         <v>0</v>
       </c>
       <c r="E74" t="n">
-        <v>1.862435268512429</v>
+        <v>1.902638697180338</v>
       </c>
       <c r="F74" t="n">
-        <v>2.310442756701851</v>
+        <v>2.407332523173834</v>
       </c>
       <c r="G74" t="n">
-        <v>-0.3953726813445599</v>
+        <v>-0.5148581110560242</v>
       </c>
       <c r="H74" t="n">
         <v>24</v>
@@ -2363,7 +2363,7 @@
         <v>45830</v>
       </c>
       <c r="B75" t="n">
-        <v>3.048692367984383</v>
+        <v>3.172570646134826</v>
       </c>
       <c r="C75" t="n">
         <v>24</v>
@@ -2372,13 +2372,13 @@
         <v>0</v>
       </c>
       <c r="E75" t="n">
-        <v>1.772006915925337</v>
+        <v>1.847771153403495</v>
       </c>
       <c r="F75" t="n">
-        <v>2.338415644014145</v>
+        <v>2.41480657695276</v>
       </c>
       <c r="G75" t="n">
-        <v>-0.8485428131461683</v>
+        <v>-0.9712912670550029</v>
       </c>
       <c r="H75" t="n">
         <v>24</v>
@@ -2389,7 +2389,7 @@
         <v>45831</v>
       </c>
       <c r="B76" t="n">
-        <v>2.912273896525415</v>
+        <v>2.803732302173691</v>
       </c>
       <c r="C76" t="n">
         <v>24</v>
@@ -2398,13 +2398,13 @@
         <v>0</v>
       </c>
       <c r="E76" t="n">
-        <v>1.713112660276108</v>
+        <v>1.64669453170847</v>
       </c>
       <c r="F76" t="n">
-        <v>2.041227990093917</v>
+        <v>2.029867882807511</v>
       </c>
       <c r="G76" t="n">
-        <v>-0.4130550378015141</v>
+        <v>-0.3973705691392693</v>
       </c>
       <c r="H76" t="n">
         <v>24</v>
@@ -2415,7 +2415,7 @@
         <v>45832</v>
       </c>
       <c r="B77" t="n">
-        <v>3.462298274661694</v>
+        <v>3.37262622526623</v>
       </c>
       <c r="C77" t="n">
         <v>24</v>
@@ -2424,13 +2424,13 @@
         <v>0</v>
       </c>
       <c r="E77" t="n">
-        <v>1.993305884280669</v>
+        <v>1.94700830814323</v>
       </c>
       <c r="F77" t="n">
-        <v>2.827016049545562</v>
+        <v>2.836694090304411</v>
       </c>
       <c r="G77" t="n">
-        <v>-0.4802395339275449</v>
+        <v>-0.4903918216263012</v>
       </c>
       <c r="H77" t="n">
         <v>24</v>
@@ -2441,7 +2441,7 @@
         <v>45833</v>
       </c>
       <c r="B78" t="n">
-        <v>2.974129980659721</v>
+        <v>2.71827227006436</v>
       </c>
       <c r="C78" t="n">
         <v>24</v>
@@ -2450,13 +2450,13 @@
         <v>0</v>
       </c>
       <c r="E78" t="n">
-        <v>1.624068378572489</v>
+        <v>1.484142272982241</v>
       </c>
       <c r="F78" t="n">
-        <v>2.293095802383385</v>
+        <v>2.163615513535983</v>
       </c>
       <c r="G78" t="n">
-        <v>0.6700819936840354</v>
+        <v>0.7062879300342881</v>
       </c>
       <c r="H78" t="n">
         <v>24</v>
@@ -2467,7 +2467,7 @@
         <v>45834</v>
       </c>
       <c r="B79" t="n">
-        <v>2.56839780357964</v>
+        <v>2.394276153909532</v>
       </c>
       <c r="C79" t="n">
         <v>24</v>
@@ -2476,13 +2476,13 @@
         <v>0</v>
       </c>
       <c r="E79" t="n">
-        <v>1.445046900076125</v>
+        <v>1.341372312375987</v>
       </c>
       <c r="F79" t="n">
-        <v>1.949241033503247</v>
+        <v>1.792635477074829</v>
       </c>
       <c r="G79" t="n">
-        <v>0.7389363978619792</v>
+        <v>0.7791999283891675</v>
       </c>
       <c r="H79" t="n">
         <v>24</v>
@@ -2493,7 +2493,7 @@
         <v>45835</v>
       </c>
       <c r="B80" t="n">
-        <v>2.819010245660977</v>
+        <v>2.998847522019934</v>
       </c>
       <c r="C80" t="n">
         <v>24</v>
@@ -2502,13 +2502,13 @@
         <v>0</v>
       </c>
       <c r="E80" t="n">
-        <v>1.641704424977912</v>
+        <v>1.754907229719837</v>
       </c>
       <c r="F80" t="n">
-        <v>2.268291600061413</v>
+        <v>2.238109392769386</v>
       </c>
       <c r="G80" t="n">
-        <v>-0.3702731592402511</v>
+        <v>-0.3340496756918123</v>
       </c>
       <c r="H80" t="n">
         <v>24</v>
@@ -2519,7 +2519,7 @@
         <v>45836</v>
       </c>
       <c r="B81" t="n">
-        <v>2.062378086467528</v>
+        <v>2.201200716712356</v>
       </c>
       <c r="C81" t="n">
         <v>24</v>
@@ -2528,13 +2528,13 @@
         <v>0</v>
       </c>
       <c r="E81" t="n">
-        <v>1.206679664872994</v>
+        <v>1.293294412822292</v>
       </c>
       <c r="F81" t="n">
-        <v>1.638634186439306</v>
+        <v>1.674121561599699</v>
       </c>
       <c r="G81" t="n">
-        <v>0.118322529359036</v>
+        <v>0.07972059969878975</v>
       </c>
       <c r="H81" t="n">
         <v>24</v>
@@ -2545,7 +2545,7 @@
         <v>45837</v>
       </c>
       <c r="B82" t="n">
-        <v>3.295451386524876</v>
+        <v>3.392655298599175</v>
       </c>
       <c r="C82" t="n">
         <v>24</v>
@@ -2554,13 +2554,13 @@
         <v>0</v>
       </c>
       <c r="E82" t="n">
-        <v>1.906578771374542</v>
+        <v>1.978384938188237</v>
       </c>
       <c r="F82" t="n">
-        <v>2.378152602195165</v>
+        <v>2.438625407027531</v>
       </c>
       <c r="G82" t="n">
-        <v>-0.2895904007633083</v>
+        <v>-0.3560089059718667</v>
       </c>
       <c r="H82" t="n">
         <v>24</v>
@@ -2571,7 +2571,7 @@
         <v>45838</v>
       </c>
       <c r="B83" t="n">
-        <v>3.792940352017163</v>
+        <v>3.689866734138482</v>
       </c>
       <c r="C83" t="n">
         <v>23</v>
@@ -2580,13 +2580,13 @@
         <v>0</v>
       </c>
       <c r="E83" t="n">
-        <v>2.187861579448449</v>
+        <v>2.133652974356711</v>
       </c>
       <c r="F83" t="n">
-        <v>3.329054563577071</v>
+        <v>3.36278873004408</v>
       </c>
       <c r="G83" t="n">
-        <v>-0.8832772993000271</v>
+        <v>-0.9216381465731069</v>
       </c>
       <c r="H83" t="n">
         <v>23</v>

</xml_diff>